<commit_message>
Refonte méthodologique : correction beta vs pairs, marge pondérée, g terminal différencié, prise de position sur écarts consensus
</commit_message>
<xml_diff>
--- a/ko_valuation_output.xlsx
+++ b/ko_valuation_output.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sommaire" sheetId="1" state="visible" r:id="rId3"/>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">Synthèse de valorisation — KO</t>
   </si>
   <si>
-    <t xml:space="preserve">Généré le 21/09/2026</t>
+    <t xml:space="preserve">Généré le 26/09/2026</t>
   </si>
   <si>
     <t xml:space="preserve">VALORISATION</t>
@@ -213,7 +213,7 @@
     <t xml:space="preserve">Marge d'EBIT</t>
   </si>
   <si>
-    <t xml:space="preserve">Moyenne des 3 derniers exercices (yfinance) (Bear/Bull = delta ± 2% vs Base)</t>
+    <t xml:space="preserve">Moyenne pondérée des 3 derniers exercices (yfinance), poids croissants vers l'exercice le plus récent (Bear/Bull = delta ± 2% vs Base)</t>
   </si>
   <si>
     <t xml:space="preserve">Croissance perpétuelle (g)</t>
@@ -1839,18 +1839,17 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+              <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                <a:uFillTx/>
+                <a:latin typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1800" b="1" u="none" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
+                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
               <a:t>Football Field</a:t>
@@ -1888,7 +1887,7 @@
           </c:tx>
           <c:spPr>
             <a:noFill/>
-            <a:ln w="0">
+            <a:ln w="12600">
               <a:noFill/>
             </a:ln>
           </c:spPr>
@@ -1899,7 +1898,8 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
@@ -1911,7 +1911,6 @@
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator> </c:separator>
-            <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
@@ -1945,16 +1944,16 @@
                 <c:formatCode>\$#,##0.00</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>34.0204935158685</c:v>
+                  <c:v>30.0244793995582</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>27.1743011272674</c:v>
+                  <c:v>26.5948941599822</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>65.35</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>87.75</c:v>
+                  <c:v>87.31</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1976,9 +1975,9 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="1f3864"/>
+              <a:srgbClr val="1F3864"/>
             </a:solidFill>
-            <a:ln w="0">
+            <a:ln w="12600">
               <a:noFill/>
             </a:ln>
           </c:spPr>
@@ -1989,7 +1988,8 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
@@ -2001,7 +2001,6 @@
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
             <c:separator> </c:separator>
-            <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
@@ -2035,10 +2034,10 @@
                 <c:formatCode>\$#,##0.00</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>53.8014181629842</c:v>
+                  <c:v>42.4461567743337</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46.3610968557609</c:v>
+                  <c:v>48.2400959480158</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>27.14</c:v>
@@ -2052,11 +2051,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="14284644"/>
-        <c:axId val="52325641"/>
+        <c:axId val="32541030"/>
+        <c:axId val="56408857"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="14284644"/>
+        <c:axId val="32541030"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2069,18 +2068,17 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                  <a:defRPr sz="1300" b="0" u="none" strike="noStrike">
+                    <a:uFillTx/>
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr sz="1000" b="1" u="none" strike="noStrike">
                     <a:solidFill>
                       <a:srgbClr val="000000"/>
                     </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
+                    <a:uFillTx/>
                     <a:latin typeface="Calibri"/>
                   </a:rPr>
                   <a:t>Valeur par action</a:t>
@@ -2113,16 +2111,17 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
+                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52325641"/>
+        <c:crossAx val="56408857"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2130,7 +2129,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52325641"/>
+        <c:axId val="56408857"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2163,21 +2162,21 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
+                <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14284644"/>
+        <c:crossAx val="32541030"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
-        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -2187,17 +2186,235 @@
     <c:dispBlanksAs val="gap"/>
   </c:chart>
   <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="ffffff"/>
-    </a:solidFill>
     <a:ln w="9360">
       <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
+        <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
   </c:spPr>
 </c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataLabel>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <cs:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointMarkerLayout>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+  </cs:wall>
+</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2206,22 +2423,22 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>160920</xdr:rowOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>162000</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="0" name="Chart 1"/>
+        <xdr:cNvPr id="1" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="6955200" y="571680"/>
+        <a:off x="6955200" y="601200"/>
         <a:ext cx="7199640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2243,34 +2460,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -2281,11 +2498,69 @@
         <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -2416,7 +2691,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B32"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
@@ -2444,7 +2719,7 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">'DCF - Modèle'!B62</f>
-        <v>88.25</v>
+        <v>87.81</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2453,7 +2728,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">'DCF - Modèle'!B61</f>
-        <v>54.2034838612625</v>
+        <v>46.7235049971412</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2471,7 +2746,7 @@
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">'Comps - Résultat'!D16</f>
-        <v>49.1509867646168</v>
+        <v>49.0382399370565</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2480,7 +2755,7 @@
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">'DCF - Modèle'!B63</f>
-        <v>0.614203783130453</v>
+        <v>0.532097767875426</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2489,7 +2764,7 @@
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">'DCF - Modèle'!B21</f>
-        <v>0.0555853234236391</v>
+        <v>0.0653502438507117</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2498,7 +2773,7 @@
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">'DCF - Modèle'!E27</f>
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2507,7 +2782,7 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">'DCF - Modèle'!E26</f>
-        <v>0.298417303761967</v>
+        <v>0.30254365140569</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2521,7 +2796,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="13" t="n">
-        <v>34.0204935158685</v>
+        <v>30.0244793995582</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2529,7 +2804,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="13" t="n">
-        <v>54.2034838612625</v>
+        <v>46.7235049971412</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2537,7 +2812,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="14" t="n">
-        <v>87.8219116788527</v>
+        <v>72.470636173892</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2652,7 +2927,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F63"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="13"/>
@@ -2704,7 +2979,7 @@
         <v>40</v>
       </c>
       <c r="B6" s="30" t="n">
-        <v>0.342</v>
+        <v>0.561166666666667</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>41</v>
@@ -2737,7 +3012,7 @@
         <v>46</v>
       </c>
       <c r="B9" s="31" t="n">
-        <v>379699.953664</v>
+        <v>377806.815232</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2761,7 +3036,7 @@
         <v>49</v>
       </c>
       <c r="B12" s="32" t="n">
-        <v>4302.549050017</v>
+        <v>4302.5488581255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2800,7 +3075,7 @@
       </c>
       <c r="B18" s="34" t="n">
         <f aca="false">B4+B6*B5</f>
-        <v>0.0591</v>
+        <v>0.0700583333333333</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2809,7 +3084,7 @@
       </c>
       <c r="B19" s="34" t="n">
         <f aca="false">B9/(B9+B10)</f>
-        <v>0.89300832339845</v>
+        <v>0.892529819685257</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2818,7 +3093,7 @@
       </c>
       <c r="B20" s="34" t="n">
         <f aca="false">1-B19</f>
-        <v>0.10699167660155</v>
+        <v>0.107470180314743</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2827,7 +3102,7 @@
       </c>
       <c r="B21" s="36" t="n">
         <f aca="false">B19*B18+B20*B7*(1-B8)</f>
-        <v>0.0555853234236391</v>
+        <v>0.0653502438507117</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2871,17 +3146,17 @@
         <v>60</v>
       </c>
       <c r="B26" s="44" t="n">
-        <v>0.278417303761967</v>
+        <v>0.28254365140569</v>
       </c>
       <c r="C26" s="44" t="n">
-        <v>0.298417303761967</v>
+        <v>0.30254365140569</v>
       </c>
       <c r="D26" s="44" t="n">
-        <v>0.318417303761967</v>
+        <v>0.32254365140569</v>
       </c>
       <c r="E26" s="45" t="n">
         <f aca="false">CHOOSE($B$24,B26,C26,D26)</f>
-        <v>0.298417303761967</v>
+        <v>0.30254365140569</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>61</v>
@@ -2892,17 +3167,17 @@
         <v>62</v>
       </c>
       <c r="B27" s="46" t="n">
-        <v>0.01</v>
+        <v>0.015</v>
       </c>
       <c r="C27" s="46" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="D27" s="46" t="n">
-        <v>0.03</v>
+        <v>0.035</v>
       </c>
       <c r="E27" s="47" t="n">
         <f aca="false">CHOOSE($B$24,B27,C27,D27)</f>
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3093,23 +3368,23 @@
       </c>
       <c r="B40" s="58" t="n">
         <f aca="false">B39*$E$26</f>
-        <v>14592.5524388455</v>
+        <v>14794.330095881</v>
       </c>
       <c r="C40" s="58" t="n">
         <f aca="false">C39*$E$26</f>
-        <v>14884.4034876224</v>
+        <v>15090.2166977986</v>
       </c>
       <c r="D40" s="58" t="n">
         <f aca="false">D39*$E$26</f>
-        <v>15107.6695399368</v>
+        <v>15316.5699482656</v>
       </c>
       <c r="E40" s="58" t="n">
         <f aca="false">E39*$E$26</f>
-        <v>15334.2845830358</v>
+        <v>15546.3184974896</v>
       </c>
       <c r="F40" s="59" t="n">
         <f aca="false">F39*$E$26</f>
-        <v>15487.6274288662</v>
+        <v>15701.7816824645</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3118,23 +3393,23 @@
       </c>
       <c r="B41" s="55" t="n">
         <f aca="false">B40*(1-$B$8)</f>
-        <v>10944.4143291341</v>
+        <v>11095.7475719107</v>
       </c>
       <c r="C41" s="55" t="n">
         <f aca="false">C40*(1-$B$8)</f>
-        <v>11163.3026157168</v>
+        <v>11317.6625233489</v>
       </c>
       <c r="D41" s="55" t="n">
         <f aca="false">D40*(1-$B$8)</f>
-        <v>11330.7521549526</v>
+        <v>11487.4274611992</v>
       </c>
       <c r="E41" s="55" t="n">
         <f aca="false">E40*(1-$B$8)</f>
-        <v>11500.7134372769</v>
+        <v>11659.7388731172</v>
       </c>
       <c r="F41" s="56" t="n">
         <f aca="false">F40*(1-$B$8)</f>
-        <v>11615.7205716496</v>
+        <v>11776.3362618483</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3218,23 +3493,23 @@
       </c>
       <c r="B45" s="60" t="n">
         <f aca="false">B41+B42-B43-B44</f>
-        <v>9721.91882913414</v>
+        <v>9873.25207191073</v>
       </c>
       <c r="C45" s="60" t="n">
         <f aca="false">C41+C42-C43-C44</f>
-        <v>9916.35720571683</v>
+        <v>10070.7171133489</v>
       </c>
       <c r="D45" s="60" t="n">
         <f aca="false">D41+D42-D43-D44</f>
-        <v>10065.1025638026</v>
+        <v>10221.7778700492</v>
       </c>
       <c r="E45" s="60" t="n">
         <f aca="false">E41+E42-E43-E44</f>
-        <v>10216.0791022596</v>
+        <v>10375.1045380999</v>
       </c>
       <c r="F45" s="61" t="n">
         <f aca="false">F41+F42-F43-F44</f>
-        <v>10318.2398932822</v>
+        <v>10478.8555834809</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3263,23 +3538,23 @@
       </c>
       <c r="B47" s="64" t="n">
         <f aca="false">1/(1+$B$21)^B46</f>
-        <v>0.947341704938303</v>
+        <v>0.938658441927508</v>
       </c>
       <c r="C47" s="64" t="n">
         <f aca="false">1/(1+$B$21)^C46</f>
-        <v>0.897456305915411</v>
+        <v>0.881079670601777</v>
       </c>
       <c r="D47" s="64" t="n">
         <f aca="false">1/(1+$B$21)^D46</f>
-        <v>0.850197786953536</v>
+        <v>0.827032870821067</v>
       </c>
       <c r="E47" s="64" t="n">
         <f aca="false">1/(1+$B$21)^E46</f>
-        <v>0.805427821027335</v>
+        <v>0.776301385947737</v>
       </c>
       <c r="F47" s="65" t="n">
         <f aca="false">1/(1+$B$21)^F46</f>
-        <v>0.763015365176778</v>
+        <v>0.728681849399868</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3288,23 +3563,23 @@
       </c>
       <c r="B48" s="67" t="n">
         <f aca="false">B45*B47</f>
-        <v>9209.97915886373</v>
+        <v>9267.61140657727</v>
       </c>
       <c r="C48" s="67" t="n">
         <f aca="false">C45*C47</f>
-        <v>8899.49730598029</v>
+        <v>8873.10411695318</v>
       </c>
       <c r="D48" s="67" t="n">
         <f aca="false">D45*D47</f>
-        <v>8557.32792520531</v>
+        <v>8453.74629676202</v>
       </c>
       <c r="E48" s="67" t="n">
         <f aca="false">E45*E47</f>
-        <v>8228.31433077586</v>
+        <v>8054.20803227962</v>
       </c>
       <c r="F48" s="68" t="n">
         <f aca="false">F45*F47</f>
-        <v>7872.97558015432</v>
+        <v>7635.75186616501</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3319,7 +3594,7 @@
       </c>
       <c r="B51" s="56" t="n">
         <f aca="false">F45*(1+E27)/(B21-E27)</f>
-        <v>295756.892971119</v>
+        <v>266189.890024134</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3328,7 +3603,7 @@
       </c>
       <c r="B52" s="69" t="n">
         <f aca="false">B51*F47</f>
-        <v>225667.053693907</v>
+        <v>193967.741354334</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3343,7 +3618,7 @@
       </c>
       <c r="B55" s="70" t="n">
         <f aca="false">SUM(B48:F48)</f>
-        <v>42768.0943009795</v>
+        <v>42284.4217187371</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3352,7 +3627,7 @@
       </c>
       <c r="B56" s="70" t="n">
         <f aca="false">B52</f>
-        <v>225667.053693907</v>
+        <v>193967.741354334</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3361,7 +3636,7 @@
       </c>
       <c r="B57" s="61" t="n">
         <f aca="false">B55+B56</f>
-        <v>268435.147994887</v>
+        <v>236252.163073071</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3379,7 +3654,7 @@
       </c>
       <c r="B59" s="61" t="n">
         <f aca="false">B57-B58</f>
-        <v>233213.147994887</v>
+        <v>201030.163073071</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3388,7 +3663,7 @@
       </c>
       <c r="B60" s="71" t="n">
         <f aca="false">B12</f>
-        <v>4302.549050017</v>
+        <v>4302.5488581255</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3397,7 +3672,7 @@
       </c>
       <c r="B61" s="72" t="n">
         <f aca="false">B59/B60</f>
-        <v>54.2034838612625</v>
+        <v>46.7235049971412</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,7 +3680,7 @@
         <v>3</v>
       </c>
       <c r="B62" s="73" t="n">
-        <v>88.25</v>
+        <v>87.81</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3414,7 +3689,7 @@
       </c>
       <c r="B63" s="74" t="n">
         <f aca="false">B61/B62</f>
-        <v>0.614203783130453</v>
+        <v>0.532097767875426</v>
       </c>
     </row>
   </sheetData>
@@ -3443,7 +3718,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="1" style="0" width="12"/>
   </cols>
@@ -3463,144 +3738,144 @@
         <v>94</v>
       </c>
       <c r="B3" s="76" t="n">
-        <v>0.01</v>
+        <v>0.015</v>
       </c>
       <c r="C3" s="76" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="D3" s="76" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="E3" s="76" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
       <c r="F3" s="76" t="n">
-        <v>0.03</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="77" t="n">
-        <v>0.0356</v>
+        <v>0.0454</v>
       </c>
       <c r="B4" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A4)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+B$3))/($A4-B$3)/(1+$A4)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>81.7616349028851</v>
+        <v>67.3276810329304</v>
       </c>
       <c r="C4" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A4)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+C$3))/($A4-C$3)/(1+$A4)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>101.530167914809</v>
+        <v>80.5321446848851</v>
       </c>
       <c r="D4" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A4)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+D$3))/($A4-D$3)/(1+$A4)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>133.970837472839</v>
+        <v>100.209384636818</v>
       </c>
       <c r="E4" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A4)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+E$3))/($A4-E$3)/(1+$A4)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>197.015912274292</v>
+        <v>132.664053128966</v>
       </c>
       <c r="F4" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A4)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+F$3))/($A4-F$3)/(1+$A4)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>372.641477792626</v>
+        <v>196.325133632796</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="77" t="n">
-        <v>0.0456</v>
+        <v>0.0554</v>
       </c>
       <c r="B5" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A5)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+B$3))/($A5-B$3)/(1+$A5)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>56.4753440866855</v>
+        <v>48.642861580274</v>
       </c>
       <c r="C5" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A5)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+C$3))/($A5-C$3)/(1+$A5)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>65.6844204083307</v>
+        <v>55.5057203584414</v>
       </c>
       <c r="D5" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A5)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+D$3))/($A5-D$3)/(1+$A5)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>78.4907921681186</v>
+        <v>64.6260984715324</v>
       </c>
       <c r="E5" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A5)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+E$3))/($A5-E$3)/(1+$A5)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>97.5138492481918</v>
+        <v>77.3371766291473</v>
       </c>
       <c r="F5" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A5)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+F$3))/($A5-F$3)/(1+$A5)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>128.731173687286</v>
+        <v>96.2791754522598</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="77" t="n">
-        <v>0.0556</v>
+        <v>0.0654</v>
       </c>
       <c r="B6" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A6)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+B$3))/($A6-B$3)/(1+$A6)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>42.2799916284506</v>
+        <v>37.3723454414473</v>
       </c>
       <c r="C6" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A6)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+C$3))/($A6-C$3)/(1+$A6)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>47.4962775993984</v>
+        <v>41.5030191423605</v>
       </c>
       <c r="D6" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A6)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+D$3))/($A6-D$3)/(1+$A6)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>54.17781243859</v>
+        <v>46.6561368286482</v>
       </c>
       <c r="E6" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A6)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+E$3))/($A6-E$3)/(1+$A6)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>63.0428553951644</v>
+        <v>53.2649374771641</v>
       </c>
       <c r="F6" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A6)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+F$3))/($A6-F$3)/(1+$A6)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>75.3708057566507</v>
+        <v>62.0476857074286</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="77" t="n">
-        <v>0.0656</v>
+        <v>0.0754</v>
       </c>
       <c r="B7" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A7)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+B$3))/($A7-B$3)/(1+$A7)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>33.1912429894393</v>
+        <v>29.8335466298767</v>
       </c>
       <c r="C7" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A7)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+C$3))/($A7-C$3)/(1+$A7)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>36.4968227388902</v>
+        <v>32.5545633897545</v>
       </c>
       <c r="D7" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A7)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+D$3))/($A7-D$3)/(1+$A7)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>40.527310328133</v>
+        <v>35.8154644273858</v>
       </c>
       <c r="E7" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A7)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+E$3))/($A7-E$3)/(1+$A7)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>45.5505288506867</v>
+        <v>39.7946256054645</v>
       </c>
       <c r="F7" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A7)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+F$3))/($A7-F$3)/(1+$A7)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>51.9847638121601</v>
+        <v>44.7587276692063</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="77" t="n">
-        <v>0.0756</v>
+        <v>0.0854</v>
       </c>
       <c r="B8" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A8)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+B$3))/($A8-B$3)/(1+$A8)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>26.873748761186</v>
+        <v>24.436256721396</v>
       </c>
       <c r="C8" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A8)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+C$3))/($A8-C$3)/(1+$A8)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>29.1273141152832</v>
+        <v>26.3419296837776</v>
       </c>
       <c r="D8" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A8)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+D$3))/($A8-D$3)/(1+$A8)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>31.7861969791101</v>
+        <v>28.5631114147654</v>
       </c>
       <c r="E8" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A8)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+E$3))/($A8-E$3)/(1+$A8)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>34.9705507646419</v>
+        <v>31.1852284762564</v>
       </c>
       <c r="F8" s="78" t="n">
         <f aca="false">IFERROR((SUMPRODUCT('DCF - Modèle'!$B$45:$F$45,1/(1+$A8)^'DCF - Modèle'!$B$46:$F$46)+('DCF - Modèle'!$F$45*(1+F$3))/($A8-F$3)/(1+$A8)^'DCF - Modèle'!$F$46-'DCF - Modèle'!$B$11)/'DCF - Modèle'!$B$12,"n/a")</f>
-        <v>38.8532277487553</v>
+        <v>34.3276068594719</v>
       </c>
     </row>
   </sheetData>
@@ -3632,7 +3907,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
@@ -3681,22 +3956,22 @@
         <v>105</v>
       </c>
       <c r="C4" s="81" t="n">
-        <v>177238.50752</v>
+        <v>175708.585984</v>
       </c>
       <c r="D4" s="81" t="n">
-        <v>219764.686848</v>
+        <v>218235.994112</v>
       </c>
       <c r="E4" s="82" t="n">
-        <v>17.005241</v>
+        <v>16.858454</v>
       </c>
       <c r="F4" s="82" t="n">
-        <v>14.456196</v>
+        <v>14.354602</v>
       </c>
       <c r="G4" s="82" t="n">
-        <v>11.639</v>
+        <v>11.558</v>
       </c>
       <c r="H4" s="82" t="n">
-        <v>2.268</v>
+        <v>2.252</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3707,22 +3982,22 @@
         <v>107</v>
       </c>
       <c r="C5" s="81" t="n">
-        <v>42131.16928</v>
+        <v>43478.392832</v>
       </c>
       <c r="D5" s="81" t="n">
-        <v>82747.170816</v>
+        <v>84094.394368</v>
       </c>
       <c r="E5" s="82" t="n">
-        <v>31.272726</v>
+        <v>32.272728</v>
       </c>
       <c r="F5" s="82" t="n">
-        <v>12.21456</v>
+        <v>12.605143</v>
       </c>
       <c r="G5" s="82" t="n">
-        <v>17.214</v>
+        <v>17.494</v>
       </c>
       <c r="H5" s="82" t="n">
-        <v>4.119</v>
+        <v>4.186</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3733,22 +4008,22 @@
         <v>109</v>
       </c>
       <c r="C6" s="81" t="n">
-        <v>87589.199872</v>
+        <v>84454.719488</v>
       </c>
       <c r="D6" s="81" t="n">
-        <v>84262.879232</v>
+        <v>81128.398848</v>
       </c>
       <c r="E6" s="82" t="n">
-        <v>41.398144</v>
+        <v>39.916664</v>
       </c>
       <c r="F6" s="82" t="n">
-        <v>34.15219</v>
+        <v>32.929512</v>
       </c>
       <c r="G6" s="82" t="n">
-        <v>28.726</v>
+        <v>27.658</v>
       </c>
       <c r="H6" s="82" t="n">
-        <v>9.14</v>
+        <v>8.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3759,22 +4034,22 @@
         <v>111</v>
       </c>
       <c r="C7" s="81" t="n">
-        <v>7090.041856</v>
+        <v>7082.450944</v>
       </c>
       <c r="D7" s="81" t="n">
-        <v>8893.632512</v>
+        <v>8886.0416</v>
       </c>
       <c r="E7" s="82" t="n">
-        <v>121.82609</v>
+        <v>121.69565</v>
       </c>
       <c r="F7" s="82" t="n">
-        <v>16.18652</v>
+        <v>16.16919</v>
       </c>
       <c r="G7" s="82" t="n">
-        <v>13.24</v>
+        <v>13.229</v>
       </c>
       <c r="H7" s="82" t="n">
-        <v>2.919</v>
+        <v>2.916</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3785,22 +4060,22 @@
         <v>113</v>
       </c>
       <c r="C8" s="81" t="n">
-        <v>2958.243584</v>
+        <v>2777.565952</v>
       </c>
       <c r="D8" s="81" t="n">
-        <v>2904.966656</v>
+        <v>2724.289024</v>
       </c>
       <c r="E8" s="82" t="n">
-        <v>16.989248</v>
+        <v>15.951612</v>
       </c>
       <c r="F8" s="82" t="n">
-        <v>16.163269</v>
+        <v>15.176083</v>
       </c>
       <c r="G8" s="82" t="n">
-        <v>12.034</v>
+        <v>11.285</v>
       </c>
       <c r="H8" s="82" t="n">
-        <v>2.46</v>
+        <v>2.307</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3811,22 +4086,22 @@
         <v>115</v>
       </c>
       <c r="C9" s="81" t="n">
-        <v>20320.59392</v>
+        <v>19408.498688</v>
       </c>
       <c r="D9" s="81" t="n">
-        <v>31045.82656</v>
+        <v>30134.007808</v>
       </c>
       <c r="E9" s="82" t="n">
-        <v>11.319695</v>
+        <v>10.821904</v>
       </c>
       <c r="F9" s="82" t="n">
-        <v>9.626907</v>
+        <v>9.247398</v>
       </c>
       <c r="G9" s="82" t="n">
-        <v>8.984</v>
+        <v>8.72</v>
       </c>
       <c r="H9" s="82" t="n">
-        <v>3.428</v>
+        <v>3.327</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3851,7 +4126,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
@@ -3907,7 +4182,7 @@
       </c>
       <c r="B9" s="86" t="n">
         <f aca="false">'DCF - Modèle'!$B$12</f>
-        <v>4302.549050017</v>
+        <v>4302.5488581255</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3930,15 +4205,15 @@
       </c>
       <c r="B13" s="82" t="n">
         <f aca="false">MEDIAN('Comps - Peers'!G:G)</f>
-        <v>12.637</v>
+        <v>12.3935</v>
       </c>
       <c r="C13" s="81" t="n">
         <f aca="false">B13*$B$5</f>
-        <v>236337.174</v>
+        <v>231783.237</v>
       </c>
       <c r="D13" s="78" t="n">
         <f aca="false">(C13-$B$8)/$B$9</f>
-        <v>46.7432611835548</v>
+        <v>45.6848355431892</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3947,15 +4222,15 @@
       </c>
       <c r="B14" s="82" t="n">
         <f aca="false">MEDIAN('Comps - Peers'!H:H)</f>
-        <v>3.1735</v>
+        <v>3.1215</v>
       </c>
       <c r="C14" s="81" t="n">
         <f aca="false">B14*$B$4</f>
-        <v>152140.7635</v>
+        <v>149647.8315</v>
       </c>
       <c r="D14" s="78" t="n">
         <f aca="false">(C14-$B$8)/$B$9</f>
-        <v>27.1743011272674</v>
+        <v>26.5948941599822</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3964,15 +4239,15 @@
       </c>
       <c r="B15" s="82" t="n">
         <f aca="false">MEDIAN('Comps - Peers'!E:E)</f>
-        <v>24.1389835</v>
+        <v>24.565591</v>
       </c>
       <c r="C15" s="81" t="n">
         <f aca="false">B15*$B$6</f>
-        <v>316389.6567345</v>
+        <v>321981.201237</v>
       </c>
       <c r="D15" s="78" t="n">
         <f aca="false">C15/$B$9</f>
-        <v>73.5353979830283</v>
+        <v>74.8349901079981</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3981,7 +4256,7 @@
       </c>
       <c r="D16" s="87" t="n">
         <f aca="false">AVERAGE(D13:D15)</f>
-        <v>49.1509867646168</v>
+        <v>49.0382399370565</v>
       </c>
     </row>
   </sheetData>
@@ -4001,7 +4276,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
@@ -4038,14 +4313,14 @@
         <v>132</v>
       </c>
       <c r="B5" s="78" t="n">
-        <v>34.0204935158685</v>
+        <v>30.0244793995582</v>
       </c>
       <c r="C5" s="78" t="n">
         <f aca="false">D5-B5</f>
-        <v>53.8014181629842</v>
+        <v>42.4461567743337</v>
       </c>
       <c r="D5" s="78" t="n">
-        <v>87.8219116788527</v>
+        <v>72.470636173892</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4053,14 +4328,14 @@
         <v>133</v>
       </c>
       <c r="B6" s="78" t="n">
-        <v>27.1743011272674</v>
+        <v>26.5948941599822</v>
       </c>
       <c r="C6" s="78" t="n">
         <f aca="false">D6-B6</f>
-        <v>46.3610968557609</v>
+        <v>48.2400959480158</v>
       </c>
       <c r="D6" s="78" t="n">
-        <v>73.5353979830283</v>
+        <v>74.8349901079981</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4083,14 +4358,14 @@
         <v>3</v>
       </c>
       <c r="B8" s="78" t="n">
-        <v>87.75</v>
+        <v>87.31</v>
       </c>
       <c r="C8" s="78" t="n">
         <f aca="false">D8-B8</f>
         <v>1</v>
       </c>
       <c r="D8" s="78" t="n">
-        <v>88.75</v>
+        <v>88.31</v>
       </c>
     </row>
   </sheetData>
@@ -4111,7 +4386,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F64"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
@@ -5206,7 +5481,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F84"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="10"/>
@@ -6664,7 +6939,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E62"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="10"/>

</xml_diff>